<commit_message>
skill v2p8(decrease TC num compared to TP, update readme) and rtm(plan mode)
</commit_message>
<xml_diff>
--- a/RTM_AI_FLTP.xlsx
+++ b/RTM_AI_FLTP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\xingchangchang\ai_evaluation\claude_code\rtm_gen\ai_cc_rtm_gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A1C8A9B-C5F0-4DE1-87AA-181EE391796E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78705821-5477-4ECF-ADCA-950CC32E44F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR-FL" sheetId="1" r:id="rId1"/>
@@ -911,7 +911,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -971,18 +971,35 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -994,26 +1011,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1301,13 +1298,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="25"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="24"/>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
@@ -1650,68 +1647,68 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A22" s="33" t="s">
+      <c r="A22" s="30" t="s">
         <v>83</v>
       </c>
-      <c r="B22" s="34"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="35"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="32"/>
     </row>
     <row r="23" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B23" s="32" t="s">
+      <c r="B23" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="25"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="24"/>
     </row>
     <row r="24" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B24" s="31" t="s">
+      <c r="B24" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="25"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="24"/>
     </row>
     <row r="25" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="25"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="24"/>
     </row>
     <row r="26" spans="1:5" ht="66.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B26" s="31" t="s">
+      <c r="B26" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="25"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="23"/>
+      <c r="E26" s="24"/>
     </row>
     <row r="27" spans="1:5" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B27" s="32" t="s">
+      <c r="B27" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="25"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="24"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A28"/>
@@ -1870,14 +1867,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="25"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="24"/>
     </row>
     <row r="2" spans="1:6" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="16" t="s">
@@ -2788,74 +2785,74 @@
       <c r="F65" s="8"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A69" s="37" t="s">
+      <c r="A69" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="B69" s="38"/>
-      <c r="C69" s="38"/>
-      <c r="D69" s="38"/>
-      <c r="E69" s="38"/>
-      <c r="F69" s="38"/>
+      <c r="B69" s="27"/>
+      <c r="C69" s="27"/>
+      <c r="D69" s="27"/>
+      <c r="E69" s="27"/>
+      <c r="F69" s="27"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A70" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="B70" s="31" t="s">
+      <c r="B70" s="22" t="s">
         <v>189</v>
       </c>
-      <c r="C70" s="24"/>
-      <c r="D70" s="24"/>
-      <c r="E70" s="24"/>
-      <c r="F70" s="25"/>
+      <c r="C70" s="23"/>
+      <c r="D70" s="23"/>
+      <c r="E70" s="23"/>
+      <c r="F70" s="24"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A71" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B71" s="31" t="s">
+      <c r="B71" s="22" t="s">
         <v>190</v>
       </c>
-      <c r="C71" s="24"/>
-      <c r="D71" s="24"/>
-      <c r="E71" s="24"/>
-      <c r="F71" s="25"/>
+      <c r="C71" s="23"/>
+      <c r="D71" s="23"/>
+      <c r="E71" s="23"/>
+      <c r="F71" s="24"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A72" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B72" s="31" t="s">
+      <c r="B72" s="22" t="s">
         <v>191</v>
       </c>
-      <c r="C72" s="24"/>
-      <c r="D72" s="24"/>
-      <c r="E72" s="24"/>
-      <c r="F72" s="25"/>
+      <c r="C72" s="23"/>
+      <c r="D72" s="23"/>
+      <c r="E72" s="23"/>
+      <c r="F72" s="24"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A73" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="B73" s="31" t="s">
+      <c r="B73" s="22" t="s">
         <v>192</v>
       </c>
-      <c r="C73" s="24"/>
-      <c r="D73" s="24"/>
-      <c r="E73" s="24"/>
-      <c r="F73" s="25"/>
+      <c r="C73" s="23"/>
+      <c r="D73" s="23"/>
+      <c r="E73" s="23"/>
+      <c r="F73" s="24"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A74" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="B74" s="31" t="s">
+      <c r="B74" s="22" t="s">
         <v>194</v>
       </c>
-      <c r="C74" s="24"/>
-      <c r="D74" s="24"/>
-      <c r="E74" s="24"/>
-      <c r="F74" s="25"/>
+      <c r="C74" s="23"/>
+      <c r="D74" s="23"/>
+      <c r="E74" s="23"/>
+      <c r="F74" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2884,20 +2881,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="29" t="s">
         <v>195</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="25"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="24"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="29" t="s">
         <v>196</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="25"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="24"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A3" s="5"/>
@@ -3073,7 +3070,7 @@
       <c r="C31" s="6"/>
       <c r="D31" s="4"/>
     </row>
-    <row r="32" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A32" s="5"/>
       <c r="B32" s="5"/>
       <c r="C32" s="6"/>
@@ -3158,44 +3155,44 @@
       <c r="D45" s="4"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A49" s="27" t="s">
+      <c r="A49" s="34" t="s">
         <v>197</v>
       </c>
-      <c r="B49" s="28"/>
-      <c r="C49" s="28"/>
-      <c r="D49" s="28"/>
+      <c r="B49" s="35"/>
+      <c r="C49" s="35"/>
+      <c r="D49" s="35"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A50" s="11" t="s">
         <v>198</v>
       </c>
-      <c r="B50" s="29" t="s">
+      <c r="B50" s="36" t="s">
         <v>199</v>
       </c>
-      <c r="C50" s="24"/>
-      <c r="D50" s="25"/>
+      <c r="C50" s="23"/>
+      <c r="D50" s="24"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A51" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="B51" s="30" t="s">
+      <c r="B51" s="37" t="s">
         <v>201</v>
       </c>
-      <c r="C51" s="24"/>
-      <c r="D51" s="25"/>
+      <c r="C51" s="23"/>
+      <c r="D51" s="24"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A52" s="11"/>
-      <c r="B52" s="23"/>
-      <c r="C52" s="24"/>
-      <c r="D52" s="25"/>
+      <c r="B52" s="33"/>
+      <c r="C52" s="23"/>
+      <c r="D52" s="24"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A53" s="11"/>
-      <c r="B53" s="23"/>
-      <c r="C53" s="24"/>
-      <c r="D53" s="25"/>
+      <c r="B53" s="33"/>
+      <c r="C53" s="23"/>
+      <c r="D53" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -3214,7 +3211,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="13.75" style="10" customWidth="1"/>
@@ -3224,12 +3221,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="25"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="24"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
@@ -3252,298 +3249,454 @@
       <c r="D3" s="4"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A4" s="21"/>
-      <c r="B4" s="21"/>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
       <c r="C4" s="3"/>
       <c r="D4" s="13"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A5" s="21"/>
-      <c r="B5" s="21"/>
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
       <c r="C5" s="3"/>
       <c r="D5" s="13"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A6" s="21"/>
-      <c r="B6" s="21"/>
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
       <c r="C6" s="3"/>
       <c r="D6" s="13"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A7" s="21"/>
-      <c r="B7" s="21"/>
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
       <c r="C7" s="3"/>
       <c r="D7" s="13"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A8" s="21"/>
-      <c r="B8" s="21"/>
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
       <c r="C8" s="3"/>
       <c r="D8" s="13"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A9" s="21"/>
-      <c r="B9" s="21"/>
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
       <c r="C9" s="3"/>
       <c r="D9" s="13"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A10" s="21"/>
-      <c r="B10" s="21"/>
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
       <c r="C10" s="3"/>
       <c r="D10" s="13"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A11" s="21"/>
-      <c r="B11" s="21"/>
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
       <c r="C11" s="3"/>
       <c r="D11" s="13"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A12" s="21"/>
-      <c r="B12" s="21"/>
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
       <c r="C12" s="3"/>
       <c r="D12" s="13"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A13" s="21"/>
-      <c r="B13" s="21"/>
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
       <c r="C13" s="3"/>
       <c r="D13" s="13"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A14" s="21"/>
-      <c r="B14" s="21"/>
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
       <c r="C14" s="3"/>
       <c r="D14" s="13"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A15" s="21"/>
-      <c r="B15" s="21"/>
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
       <c r="C15" s="3"/>
       <c r="D15" s="13"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A16" s="21"/>
-      <c r="B16" s="21"/>
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
       <c r="C16" s="3"/>
       <c r="D16" s="13"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A17" s="21"/>
-      <c r="B17" s="21"/>
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
       <c r="C17" s="3"/>
       <c r="D17" s="13"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A18" s="21"/>
-      <c r="B18" s="21"/>
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
       <c r="C18" s="3"/>
       <c r="D18" s="13"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A19" s="21"/>
-      <c r="B19" s="21"/>
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
       <c r="C19" s="3"/>
       <c r="D19" s="13"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A20" s="21"/>
-      <c r="B20" s="21"/>
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
       <c r="C20" s="3"/>
       <c r="D20" s="13"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A21" s="21"/>
-      <c r="B21" s="21"/>
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
       <c r="C21" s="3"/>
       <c r="D21" s="13"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A22" s="21"/>
-      <c r="B22" s="21"/>
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
       <c r="C22" s="3"/>
       <c r="D22" s="13"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A23" s="21"/>
-      <c r="B23" s="21"/>
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
       <c r="C23" s="3"/>
       <c r="D23" s="13"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A24" s="21"/>
-      <c r="B24" s="21"/>
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
       <c r="C24" s="3"/>
       <c r="D24" s="13"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A25" s="21"/>
-      <c r="B25" s="21"/>
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
       <c r="C25" s="3"/>
       <c r="D25" s="13"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A26" s="21"/>
-      <c r="B26" s="21"/>
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
       <c r="C26" s="3"/>
       <c r="D26" s="13"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A27" s="21"/>
-      <c r="B27" s="21"/>
-      <c r="C27" s="3"/>
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="21"/>
       <c r="D27" s="13"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A28" s="21"/>
-      <c r="B28" s="21"/>
-      <c r="C28" s="3"/>
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="21"/>
       <c r="D28" s="13"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A29" s="21"/>
-      <c r="B29" s="21"/>
-      <c r="C29" s="3"/>
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="21"/>
       <c r="D29" s="13"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A30" s="21"/>
-      <c r="B30" s="21"/>
-      <c r="C30" s="3"/>
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="21"/>
       <c r="D30" s="13"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="4"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="13"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="4"/>
+      <c r="C32" s="21"/>
+      <c r="D32" s="13"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="4"/>
+      <c r="C33" s="21"/>
+      <c r="D33" s="13"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A34" s="4"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="4"/>
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="21"/>
+      <c r="D34" s="13"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A35" s="4"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="4"/>
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="21"/>
+      <c r="D35" s="13"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="4"/>
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="13"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="4"/>
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="21"/>
+      <c r="D37" s="13"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A38" s="4"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="4"/>
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="21"/>
+      <c r="D38" s="13"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A39" s="4"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="3"/>
-      <c r="D39" s="4"/>
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="21"/>
+      <c r="D39" s="13"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A40" s="13"/>
-      <c r="B40" s="13"/>
-      <c r="C40" s="22"/>
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="21"/>
       <c r="D40" s="13"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A41" s="13"/>
-      <c r="B41" s="13"/>
-      <c r="C41" s="22"/>
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="21"/>
       <c r="D41" s="13"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A42" s="13"/>
-      <c r="B42" s="13"/>
-      <c r="C42" s="22"/>
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="21"/>
       <c r="D42" s="13"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A43" s="13"/>
-      <c r="B43" s="13"/>
-      <c r="C43" s="22"/>
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="21"/>
       <c r="D43" s="13"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A44" s="13"/>
-      <c r="B44" s="13"/>
-      <c r="C44" s="22"/>
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="21"/>
       <c r="D44" s="13"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A45" s="13"/>
-      <c r="B45" s="13"/>
-      <c r="C45" s="22"/>
+      <c r="A45" s="2"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="21"/>
       <c r="D45" s="13"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A46" s="13"/>
-      <c r="B46" s="13"/>
-      <c r="C46" s="22"/>
+      <c r="A46" s="2"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="21"/>
       <c r="D46" s="13"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A47" s="13"/>
-      <c r="B47" s="13"/>
-      <c r="C47" s="22"/>
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="21"/>
       <c r="D47" s="13"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A48" s="13"/>
-      <c r="B48" s="13"/>
-      <c r="C48" s="22"/>
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="21"/>
       <c r="D48" s="13"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A49" s="13"/>
-      <c r="B49" s="13"/>
-      <c r="C49" s="22"/>
+      <c r="A49" s="2"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="21"/>
       <c r="D49" s="13"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A50" s="13"/>
-      <c r="B50" s="13"/>
-      <c r="C50" s="22"/>
+      <c r="A50" s="2"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="21"/>
       <c r="D50" s="13"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A51" s="13"/>
-      <c r="B51" s="13"/>
-      <c r="C51" s="22"/>
-      <c r="D51" s="15"/>
+      <c r="A51" s="2"/>
+      <c r="B51" s="2"/>
+      <c r="C51" s="21"/>
+      <c r="D51" s="13"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A52" s="13"/>
-      <c r="B52" s="13"/>
-      <c r="C52" s="22"/>
-      <c r="D52" s="15"/>
+      <c r="A52" s="2"/>
+      <c r="B52" s="2"/>
+      <c r="C52" s="21"/>
+      <c r="D52" s="13"/>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A53" s="2"/>
+      <c r="B53" s="2"/>
+      <c r="C53" s="3"/>
+      <c r="D53" s="13"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A54" s="2"/>
+      <c r="B54" s="2"/>
+      <c r="C54" s="3"/>
+      <c r="D54" s="13"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A55" s="2"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="3"/>
+      <c r="D55" s="13"/>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A56" s="2"/>
+      <c r="B56" s="2"/>
+      <c r="C56" s="3"/>
+      <c r="D56" s="13"/>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="4"/>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A58" s="2"/>
+      <c r="B58" s="2"/>
+      <c r="C58" s="3"/>
+      <c r="D58" s="4"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A59" s="2"/>
+      <c r="B59" s="2"/>
+      <c r="C59" s="3"/>
+      <c r="D59" s="4"/>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A60" s="2"/>
+      <c r="B60" s="2"/>
+      <c r="C60" s="3"/>
+      <c r="D60" s="4"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="3"/>
+      <c r="D61" s="4"/>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A62" s="2"/>
+      <c r="B62" s="2"/>
+      <c r="C62" s="3"/>
+      <c r="D62" s="4"/>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A63" s="2"/>
+      <c r="B63" s="2"/>
+      <c r="C63" s="3"/>
+      <c r="D63" s="4"/>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A64" s="2"/>
+      <c r="B64" s="2"/>
+      <c r="C64" s="3"/>
+      <c r="D64" s="4"/>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A65" s="2"/>
+      <c r="B65" s="2"/>
+      <c r="C65" s="3"/>
+      <c r="D65" s="4"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A66" s="2"/>
+      <c r="B66" s="2"/>
+      <c r="C66" s="21"/>
+      <c r="D66" s="13"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A67" s="2"/>
+      <c r="B67" s="2"/>
+      <c r="C67" s="21"/>
+      <c r="D67" s="13"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A68" s="2"/>
+      <c r="B68" s="2"/>
+      <c r="C68" s="21"/>
+      <c r="D68" s="13"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A69" s="2"/>
+      <c r="B69" s="2"/>
+      <c r="C69" s="21"/>
+      <c r="D69" s="13"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A70" s="2"/>
+      <c r="B70" s="2"/>
+      <c r="C70" s="21"/>
+      <c r="D70" s="13"/>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A71" s="2"/>
+      <c r="B71" s="2"/>
+      <c r="C71" s="21"/>
+      <c r="D71" s="13"/>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A72" s="2"/>
+      <c r="B72" s="2"/>
+      <c r="C72" s="21"/>
+      <c r="D72" s="13"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A73" s="2"/>
+      <c r="B73" s="2"/>
+      <c r="C73" s="21"/>
+      <c r="D73" s="13"/>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A74" s="2"/>
+      <c r="B74" s="2"/>
+      <c r="C74" s="21"/>
+      <c r="D74" s="13"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A75" s="2"/>
+      <c r="B75" s="2"/>
+      <c r="C75" s="21"/>
+      <c r="D75" s="13"/>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A76" s="2"/>
+      <c r="B76" s="2"/>
+      <c r="C76" s="21"/>
+      <c r="D76" s="13"/>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A77" s="2"/>
+      <c r="B77" s="2"/>
+      <c r="C77" s="21"/>
+      <c r="D77" s="15"/>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A78" s="2"/>
+      <c r="B78" s="2"/>
+      <c r="C78" s="21"/>
+      <c r="D78" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>